<commit_message>
Update Confronto Metriche - 23-5-26.xlsx
</commit_message>
<xml_diff>
--- a/PythonProject/results/Confronto Metriche - 23-5-26.xlsx
+++ b/PythonProject/results/Confronto Metriche - 23-5-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t_789\Desktop\Sviluppo\ML_4_VIsion_-_Multimedia\PythonProject\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B59AD9-FF3E-4A78-A87B-D17293AECD9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A66DDA-0896-4F3E-A71E-23598C7C67B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="161">
   <si>
     <t>LogoDet-3K</t>
   </si>
@@ -84,9 +84,6 @@
     <t>0.861679454390452</t>
   </si>
   <si>
-    <t>Dataset</t>
-  </si>
-  <si>
     <t>Loss</t>
   </si>
   <si>
@@ -475,6 +472,42 @@
   </si>
   <si>
     <t>0.7007194273161473</t>
+  </si>
+  <si>
+    <t>Dataset - M05 - LR000000003</t>
+  </si>
+  <si>
+    <t>Dataset - M05 - LR00000000003</t>
+  </si>
+  <si>
+    <t>0.7708435246875202</t>
+  </si>
+  <si>
+    <t>0.08591801045869274</t>
+  </si>
+  <si>
+    <t>0.5810791551608009</t>
+  </si>
+  <si>
+    <t>0.9469278812763072</t>
+  </si>
+  <si>
+    <t>0.8540000000000002</t>
+  </si>
+  <si>
+    <t>0.14139242585082454</t>
+  </si>
+  <si>
+    <t>0.23497592205568882</t>
+  </si>
+  <si>
+    <t>0.5311034711155903</t>
+  </si>
+  <si>
+    <t>0.6282543058149747</t>
+  </si>
+  <si>
+    <t>0.7007807462881804</t>
   </si>
 </sst>
 </file>
@@ -804,10 +837,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="18.54296875" bestFit="1" customWidth="1"/>
@@ -820,46 +853,46 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
@@ -948,46 +981,46 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="Q5" s="1"/>
     </row>
@@ -1000,13 +1033,13 @@
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>14</v>
@@ -1015,22 +1048,22 @@
         <v>15</v>
       </c>
       <c r="I6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="Q6" s="1"/>
     </row>
@@ -1042,40 +1075,40 @@
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="M7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="Q7" s="1"/>
     </row>
@@ -1097,46 +1130,46 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>31</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>32</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>33</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>34</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>35</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>36</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>37</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>38</v>
-      </c>
-      <c r="N9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
@@ -1147,37 +1180,37 @@
         <v>12</v>
       </c>
       <c r="D10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
-        <v>62</v>
-      </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G10" t="s">
         <v>14</v>
       </c>
       <c r="H10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I10" t="s">
         <v>42</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>43</v>
       </c>
-      <c r="J10" t="s">
-        <v>44</v>
-      </c>
       <c r="K10" t="s">
+        <v>62</v>
+      </c>
+      <c r="L10" t="s">
         <v>63</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>64</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>65</v>
-      </c>
-      <c r="N10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
@@ -1188,40 +1221,40 @@
         <v>12</v>
       </c>
       <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" t="s">
         <v>67</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>68</v>
-      </c>
-      <c r="E11" t="s">
-        <v>69</v>
       </c>
       <c r="F11" t="s">
         <v>4</v>
       </c>
       <c r="G11" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" t="s">
         <v>70</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J11" t="s">
         <v>71</v>
       </c>
-      <c r="I11" t="s">
-        <v>54</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>72</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>73</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>74</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>75</v>
-      </c>
-      <c r="N11" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
@@ -1232,37 +1265,37 @@
         <v>13</v>
       </c>
       <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
         <v>77</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" t="s">
         <v>78</v>
       </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12" t="s">
         <v>42</v>
       </c>
-      <c r="G12" t="s">
-        <v>79</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>80</v>
       </c>
-      <c r="I12" t="s">
-        <v>43</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>81</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>82</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>83</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>84</v>
-      </c>
-      <c r="N12" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
@@ -1273,84 +1306,84 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" t="s">
         <v>86</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>87</v>
-      </c>
-      <c r="E13" t="s">
-        <v>88</v>
       </c>
       <c r="F13" t="s">
         <v>4</v>
       </c>
       <c r="G13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" t="s">
         <v>89</v>
       </c>
-      <c r="I13" t="s">
-        <v>54</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>90</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>91</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>92</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>93</v>
-      </c>
-      <c r="N13" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" t="s">
         <v>30</v>
       </c>
-      <c r="C15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>31</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>32</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>33</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>34</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>35</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>36</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>37</v>
       </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>38</v>
-      </c>
-      <c r="N15" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.35">
@@ -1361,37 +1394,37 @@
         <v>12</v>
       </c>
       <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
         <v>96</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" t="s">
         <v>97</v>
       </c>
-      <c r="F16" t="s">
+      <c r="I16" t="s">
         <v>42</v>
       </c>
-      <c r="G16" t="s">
-        <v>42</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="J16" t="s">
         <v>98</v>
       </c>
-      <c r="I16" t="s">
-        <v>43</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>99</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>100</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>101</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>102</v>
-      </c>
-      <c r="N16" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
@@ -1402,84 +1435,84 @@
         <v>12</v>
       </c>
       <c r="C17" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" t="s">
         <v>104</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>105</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>106</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>107</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>108</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>109</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>110</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>111</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>112</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>113</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>114</v>
-      </c>
-      <c r="N17" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" t="s">
         <v>30</v>
       </c>
-      <c r="C19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>31</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>32</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>33</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>34</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>35</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>36</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>37</v>
       </c>
-      <c r="M19" t="s">
+      <c r="N19" t="s">
         <v>38</v>
-      </c>
-      <c r="N19" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
@@ -1490,37 +1523,37 @@
         <v>12</v>
       </c>
       <c r="D20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" t="s">
         <v>117</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>41</v>
+      </c>
+      <c r="G20" t="s">
         <v>118</v>
       </c>
-      <c r="F20" t="s">
+      <c r="H20" t="s">
+        <v>119</v>
+      </c>
+      <c r="I20" t="s">
         <v>42</v>
       </c>
-      <c r="G20" t="s">
-        <v>119</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="J20" t="s">
         <v>120</v>
       </c>
-      <c r="I20" t="s">
-        <v>43</v>
-      </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>121</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>122</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>123</v>
       </c>
-      <c r="M20" t="s">
+      <c r="N20" t="s">
         <v>124</v>
-      </c>
-      <c r="N20" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
@@ -1531,84 +1564,84 @@
         <v>12</v>
       </c>
       <c r="C21" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" t="s">
         <v>126</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>127</v>
-      </c>
-      <c r="E21" t="s">
-        <v>128</v>
       </c>
       <c r="F21" t="s">
         <v>4</v>
       </c>
       <c r="G21" t="s">
+        <v>128</v>
+      </c>
+      <c r="H21" t="s">
         <v>129</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
+        <v>53</v>
+      </c>
+      <c r="J21" t="s">
         <v>130</v>
       </c>
-      <c r="I21" t="s">
-        <v>54</v>
-      </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>131</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>132</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>133</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>134</v>
-      </c>
-      <c r="N21" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>149</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
         <v>19</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" t="s">
         <v>30</v>
       </c>
-      <c r="C23" t="s">
-        <v>20</v>
-      </c>
-      <c r="D23" t="s">
-        <v>21</v>
-      </c>
-      <c r="E23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>31</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>32</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>33</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>34</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>35</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>36</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>37</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>38</v>
-      </c>
-      <c r="N23" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
@@ -1619,10 +1652,10 @@
         <v>12</v>
       </c>
       <c r="D24" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" t="s">
         <v>137</v>
-      </c>
-      <c r="E24" t="s">
-        <v>138</v>
       </c>
       <c r="F24" t="s">
         <v>13</v>
@@ -1634,19 +1667,19 @@
         <v>15</v>
       </c>
       <c r="I24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J24" t="s">
+        <v>43</v>
+      </c>
+      <c r="K24" t="s">
         <v>44</v>
-      </c>
-      <c r="K24" t="s">
-        <v>45</v>
       </c>
       <c r="L24" t="s">
         <v>16</v>
       </c>
       <c r="M24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N24" t="s">
         <v>18</v>
@@ -1660,40 +1693,169 @@
         <v>12</v>
       </c>
       <c r="C25" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" t="s">
         <v>141</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>142</v>
-      </c>
-      <c r="E25" t="s">
-        <v>143</v>
       </c>
       <c r="F25" t="s">
         <v>4</v>
       </c>
       <c r="G25" t="s">
+        <v>143</v>
+      </c>
+      <c r="H25" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" t="s">
+        <v>53</v>
+      </c>
+      <c r="J25" t="s">
         <v>144</v>
       </c>
-      <c r="H25" t="s">
+      <c r="K25" t="s">
+        <v>145</v>
+      </c>
+      <c r="L25" t="s">
+        <v>146</v>
+      </c>
+      <c r="M25" t="s">
+        <v>147</v>
+      </c>
+      <c r="N25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>150</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
+        <v>31</v>
+      </c>
+      <c r="H27" t="s">
+        <v>32</v>
+      </c>
+      <c r="I27" t="s">
+        <v>33</v>
+      </c>
+      <c r="J27" t="s">
+        <v>34</v>
+      </c>
+      <c r="K27" t="s">
+        <v>35</v>
+      </c>
+      <c r="L27" t="s">
+        <v>36</v>
+      </c>
+      <c r="M27" t="s">
+        <v>37</v>
+      </c>
+      <c r="N27" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28">
+        <v>13</v>
+      </c>
+      <c r="D28" t="s">
+        <v>151</v>
+      </c>
+      <c r="E28" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I28" t="s">
+        <v>138</v>
+      </c>
+      <c r="J28" t="s">
+        <v>43</v>
+      </c>
+      <c r="K28" t="s">
+        <v>44</v>
+      </c>
+      <c r="L28" t="s">
+        <v>16</v>
+      </c>
+      <c r="M28" t="s">
+        <v>139</v>
+      </c>
+      <c r="N28" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29">
+        <v>13</v>
+      </c>
+      <c r="C29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D29" t="s">
+        <v>153</v>
+      </c>
+      <c r="E29" t="s">
+        <v>154</v>
+      </c>
+      <c r="F29" t="s">
+        <v>4</v>
+      </c>
+      <c r="G29" t="s">
+        <v>155</v>
+      </c>
+      <c r="H29" t="s">
+        <v>6</v>
+      </c>
+      <c r="I29" t="s">
         <v>53</v>
       </c>
-      <c r="I25" t="s">
-        <v>54</v>
-      </c>
-      <c r="J25" t="s">
-        <v>145</v>
-      </c>
-      <c r="K25" t="s">
-        <v>146</v>
-      </c>
-      <c r="L25" t="s">
-        <v>147</v>
-      </c>
-      <c r="M25" t="s">
-        <v>148</v>
-      </c>
-      <c r="N25" t="s">
-        <v>149</v>
+      <c r="J29" t="s">
+        <v>156</v>
+      </c>
+      <c r="K29" t="s">
+        <v>157</v>
+      </c>
+      <c r="L29" t="s">
+        <v>158</v>
+      </c>
+      <c r="M29" t="s">
+        <v>159</v>
+      </c>
+      <c r="N29" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>